<commit_message>
results run 5.1 new
</commit_message>
<xml_diff>
--- a/Development AG/new_results/run_v5.1/summary_regression_stats.xlsx
+++ b/Development AG/new_results/run_v5.1/summary_regression_stats.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="sis" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="oks" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ohs" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -513,46 +514,46 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.0178</v>
+        <v>2.4149</v>
       </c>
       <c r="C2" t="n">
-        <v>1.0244</v>
+        <v>1.1718</v>
       </c>
       <c r="D2" t="n">
-        <v>6.1739</v>
+        <v>8.5032</v>
       </c>
       <c r="E2" t="n">
-        <v>5.1639</v>
+        <v>6.6032</v>
       </c>
       <c r="F2" t="n">
-        <v>2.2575</v>
+        <v>2.6641</v>
       </c>
       <c r="G2" t="n">
-        <v>1.0682</v>
+        <v>1.2199</v>
       </c>
       <c r="H2" t="n">
-        <v>-5.7269</v>
+        <v>-10.5881</v>
       </c>
       <c r="I2" t="n">
-        <v>13.1347</v>
+        <v>22.5182</v>
       </c>
       <c r="J2" t="n">
-        <v>0.09229999999999999</v>
+        <v>0.1086</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0581</v>
+        <v>0.0618</v>
       </c>
       <c r="L2" t="n">
-        <v>1.9782</v>
+        <v>2.318</v>
       </c>
       <c r="M2" t="n">
-        <v>1.0951</v>
+        <v>1.2262</v>
       </c>
       <c r="N2" t="n">
-        <v>0.6216</v>
+        <v>0.223</v>
       </c>
       <c r="O2" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.3961</v>
       </c>
     </row>
     <row r="3">
@@ -562,46 +563,46 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.967</v>
+        <v>2.3775</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9808</v>
+        <v>1.1601</v>
       </c>
       <c r="D3" t="n">
-        <v>5.8196</v>
+        <v>8.151300000000001</v>
       </c>
       <c r="E3" t="n">
-        <v>4.6925</v>
+        <v>6.4741</v>
       </c>
       <c r="F3" t="n">
-        <v>2.1998</v>
+        <v>2.6111</v>
       </c>
       <c r="G3" t="n">
-        <v>1.0189</v>
+        <v>1.1883</v>
       </c>
       <c r="H3" t="n">
-        <v>-5.3863</v>
+        <v>-10.406</v>
       </c>
       <c r="I3" t="n">
-        <v>12.277</v>
+        <v>22.3989</v>
       </c>
       <c r="J3" t="n">
-        <v>0.0897</v>
+        <v>0.1068</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0548</v>
+        <v>0.0608</v>
       </c>
       <c r="L3" t="n">
-        <v>1.9113</v>
+        <v>2.2704</v>
       </c>
       <c r="M3" t="n">
-        <v>1.0346</v>
+        <v>1.1807</v>
       </c>
       <c r="N3" t="n">
-        <v>0.6345</v>
+        <v>0.2563</v>
       </c>
       <c r="O3" t="n">
-        <v>0.1049</v>
+        <v>0.4266</v>
       </c>
     </row>
     <row r="4">
@@ -632,28 +633,28 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3.4741</v>
+        <v>3.474</v>
       </c>
       <c r="C5" t="n">
-        <v>1.6046</v>
+        <v>1.6043</v>
       </c>
       <c r="D5" t="n">
-        <v>17.9404</v>
+        <v>17.9386</v>
       </c>
       <c r="E5" t="n">
-        <v>14.4664</v>
+        <v>14.4622</v>
       </c>
       <c r="F5" t="n">
-        <v>3.9177</v>
+        <v>3.9175</v>
       </c>
       <c r="G5" t="n">
-        <v>1.6567</v>
+        <v>1.6565</v>
       </c>
       <c r="H5" t="n">
-        <v>-17.9845</v>
+        <v>-17.9833</v>
       </c>
       <c r="I5" t="n">
-        <v>34.2192</v>
+        <v>34.2167</v>
       </c>
       <c r="J5" t="n">
         <v>0.1582</v>
@@ -665,13 +666,13 @@
         <v>3.4216</v>
       </c>
       <c r="M5" t="n">
-        <v>1.7447</v>
+        <v>1.7445</v>
       </c>
       <c r="N5" t="n">
-        <v>-1.8873</v>
+        <v>-1.8874</v>
       </c>
       <c r="O5" t="n">
-        <v>3.059</v>
+        <v>3.0598</v>
       </c>
     </row>
   </sheetData>
@@ -772,46 +773,46 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5.2275</v>
+        <v>5.8517</v>
       </c>
       <c r="C2" t="n">
-        <v>3.4001</v>
+        <v>3.8912</v>
       </c>
       <c r="D2" t="n">
-        <v>41.6557</v>
+        <v>52.9193</v>
       </c>
       <c r="E2" t="n">
-        <v>42.6563</v>
+        <v>53.0663</v>
       </c>
       <c r="F2" t="n">
-        <v>5.6149</v>
+        <v>6.2975</v>
       </c>
       <c r="G2" t="n">
-        <v>3.2748</v>
+        <v>3.7471</v>
       </c>
       <c r="H2" t="n">
-        <v>-6.3775</v>
+        <v>-8.9499</v>
       </c>
       <c r="I2" t="n">
-        <v>10.4778</v>
+        <v>13.9442</v>
       </c>
       <c r="J2" t="n">
-        <v>0.1892</v>
+        <v>0.2145</v>
       </c>
       <c r="K2" t="n">
-        <v>0.1226</v>
+        <v>0.1513</v>
       </c>
       <c r="L2" t="n">
-        <v>5.0225</v>
+        <v>5.6999</v>
       </c>
       <c r="M2" t="n">
-        <v>3.5014</v>
+        <v>4.1091</v>
       </c>
       <c r="N2" t="n">
-        <v>0.5648</v>
+        <v>0.3173</v>
       </c>
       <c r="O2" t="n">
-        <v>0.2113</v>
+        <v>0.3595</v>
       </c>
     </row>
     <row r="3">
@@ -821,46 +822,46 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5.1351</v>
+        <v>5.7406</v>
       </c>
       <c r="C3" t="n">
-        <v>3.3042</v>
+        <v>3.7553</v>
       </c>
       <c r="D3" t="n">
-        <v>40.1688</v>
+        <v>50.2518</v>
       </c>
       <c r="E3" t="n">
-        <v>40.6769</v>
+        <v>48.4934</v>
       </c>
       <c r="F3" t="n">
-        <v>5.5327</v>
+        <v>6.1505</v>
       </c>
       <c r="G3" t="n">
-        <v>3.1813</v>
+        <v>3.6269</v>
       </c>
       <c r="H3" t="n">
-        <v>-6.1716</v>
+        <v>-8.3188</v>
       </c>
       <c r="I3" t="n">
-        <v>10.2121</v>
+        <v>13.3014</v>
       </c>
       <c r="J3" t="n">
-        <v>0.1865</v>
+        <v>0.2123</v>
       </c>
       <c r="K3" t="n">
-        <v>0.1199</v>
+        <v>0.1518</v>
       </c>
       <c r="L3" t="n">
-        <v>4.9916</v>
+        <v>5.6031</v>
       </c>
       <c r="M3" t="n">
-        <v>3.5554</v>
+        <v>3.9888</v>
       </c>
       <c r="N3" t="n">
-        <v>0.5079</v>
+        <v>0.3256</v>
       </c>
       <c r="O3" t="n">
-        <v>0.2056</v>
+        <v>0.3617</v>
       </c>
     </row>
     <row r="4">
@@ -891,16 +892,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8.205399999999999</v>
+        <v>8.205500000000001</v>
       </c>
       <c r="C5" t="n">
         <v>5.4817</v>
       </c>
       <c r="D5" t="n">
-        <v>103.1101</v>
+        <v>103.112</v>
       </c>
       <c r="E5" t="n">
-        <v>115.2699</v>
+        <v>115.2712</v>
       </c>
       <c r="F5" t="n">
         <v>8.769500000000001</v>
@@ -909,10 +910,10 @@
         <v>5.2677</v>
       </c>
       <c r="H5" t="n">
-        <v>-16.7375</v>
+        <v>-16.7379</v>
       </c>
       <c r="I5" t="n">
-        <v>23.7559</v>
+        <v>23.7566</v>
       </c>
       <c r="J5" t="n">
         <v>0.2862</v>
@@ -921,7 +922,7 @@
         <v>0.1698</v>
       </c>
       <c r="L5" t="n">
-        <v>8.150499999999999</v>
+        <v>8.150600000000001</v>
       </c>
       <c r="M5" t="n">
         <v>5.7875</v>
@@ -931,6 +932,265 @@
       </c>
       <c r="O5" t="n">
         <v>0.1959</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>MAE_mean</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>MAE_std</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>MSE_mean</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>MSE_std</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>RMSE_mean</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>RMSE_std</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>R2_mean</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>R2_std</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>MAPE_mean</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>MAPE_std</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>MEDAE_mean</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>MEDAE_std</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>EVS_mean</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>EVS_std</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4.8809</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3.1704</v>
+      </c>
+      <c r="D2" t="n">
+        <v>38.4178</v>
+      </c>
+      <c r="E2" t="n">
+        <v>43.7888</v>
+      </c>
+      <c r="F2" t="n">
+        <v>5.3704</v>
+      </c>
+      <c r="G2" t="n">
+        <v>3.1843</v>
+      </c>
+      <c r="H2" t="n">
+        <v>-9.2639</v>
+      </c>
+      <c r="I2" t="n">
+        <v>17.3436</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.1876</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.1205</v>
+      </c>
+      <c r="L2" t="n">
+        <v>4.6184</v>
+      </c>
+      <c r="M2" t="n">
+        <v>3.2754</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.1559</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.306</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>LightGBM</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4.8836</v>
+      </c>
+      <c r="C3" t="n">
+        <v>3.1069</v>
+      </c>
+      <c r="D3" t="n">
+        <v>37.8158</v>
+      </c>
+      <c r="E3" t="n">
+        <v>42.9852</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5.3468</v>
+      </c>
+      <c r="G3" t="n">
+        <v>3.1258</v>
+      </c>
+      <c r="H3" t="n">
+        <v>-9.2316</v>
+      </c>
+      <c r="I3" t="n">
+        <v>17.1197</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.1874</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.1168</v>
+      </c>
+      <c r="L3" t="n">
+        <v>4.6743</v>
+      </c>
+      <c r="M3" t="n">
+        <v>3.2256</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.1979</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.2192</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>SVR</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>6.2495</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4.7695</v>
+      </c>
+      <c r="D5" t="n">
+        <v>67.6827</v>
+      </c>
+      <c r="E5" t="n">
+        <v>86.2914</v>
+      </c>
+      <c r="F5" t="n">
+        <v>6.8095</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4.7504</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-16.5904</v>
+      </c>
+      <c r="I5" t="n">
+        <v>31.6577</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.2327</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.1606</v>
+      </c>
+      <c r="L5" t="n">
+        <v>6.1391</v>
+      </c>
+      <c r="M5" t="n">
+        <v>4.8967</v>
+      </c>
+      <c r="N5" t="n">
+        <v>-0.158</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.3779</v>
       </c>
     </row>
   </sheetData>

</xml_diff>